<commit_message>
Cap nhat diem danh cuoi buoi 3
</commit_message>
<xml_diff>
--- a/DA24TTA-To2-220236.xlsx
+++ b/DA24TTA-To2-220236.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\my-project-da24tta\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tkw\my-project-da24tta\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="93">
   <si>
     <t>Đại học Trà Vinh</t>
   </si>
@@ -93,9 +93,6 @@
     <t>Tên lớp</t>
   </si>
   <si>
-    <t>Email</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
@@ -114,9 +111,6 @@
     <t>ĐH Công nghệ thông tin A 2024</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>2</t>
   </si>
   <si>
@@ -147,9 +141,6 @@
     <t>Chi</t>
   </si>
   <si>
-    <t>110124012@st.tvu.edu.vn</t>
-  </si>
-  <si>
     <t>5</t>
   </si>
   <si>
@@ -162,9 +153,6 @@
     <t>Chiến</t>
   </si>
   <si>
-    <t>110124013@st.tvu.edu.vn</t>
-  </si>
-  <si>
     <t>6</t>
   </si>
   <si>
@@ -189,9 +177,6 @@
     <t>Định</t>
   </si>
   <si>
-    <t>110124034@st.tvu.edu.vn</t>
-  </si>
-  <si>
     <t>8</t>
   </si>
   <si>
@@ -204,9 +189,6 @@
     <t>Khải</t>
   </si>
   <si>
-    <t>110124081@st.tvu.edu.vn</t>
-  </si>
-  <si>
     <t>9</t>
   </si>
   <si>
@@ -219,9 +201,6 @@
     <t>Khoa</t>
   </si>
   <si>
-    <t>110124096@st.tvu.edu.vn</t>
-  </si>
-  <si>
     <t>10</t>
   </si>
   <si>
@@ -231,9 +210,6 @@
     <t>Trần Đăng</t>
   </si>
   <si>
-    <t>110124097@st.tvu.edu.vn</t>
-  </si>
-  <si>
     <t>11</t>
   </si>
   <si>
@@ -282,9 +258,6 @@
     <t>Phước</t>
   </si>
   <si>
-    <t>110124152@st.tvu.edu.vn</t>
-  </si>
-  <si>
     <t>15</t>
   </si>
   <si>
@@ -309,9 +282,6 @@
     <t>Thành</t>
   </si>
   <si>
-    <t>110124169@st.tvu.edu.vn</t>
-  </si>
-  <si>
     <t>17</t>
   </si>
   <si>
@@ -321,13 +291,13 @@
     <t>Võ Bá</t>
   </si>
   <si>
-    <t>110124170@st.tvu.edu.vn</t>
-  </si>
-  <si>
     <t>Buổi thực hành 1</t>
   </si>
   <si>
     <t>15'</t>
+  </si>
+  <si>
+    <t>Buổi thực hành 2</t>
   </si>
 </sst>
 </file>
@@ -459,7 +429,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -473,6 +443,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -480,12 +456,10 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -839,40 +813,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="G1" s="5" t="s">
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="G1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="5"/>
+      <c r="H1" s="7"/>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="G2" s="5" t="s">
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="G2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="5"/>
+      <c r="H2" s="7"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="D4" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
+      <c r="D4" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
     </row>
     <row r="5" spans="1:9">
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
     </row>
     <row r="7" spans="1:9">
       <c r="B7" s="1" t="s">
@@ -935,64 +909,62 @@
       <c r="F11" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G11" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="H11" s="7"/>
+      <c r="G11" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H11" s="9"/>
       <c r="I11" s="2" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>28</v>
-      </c>
       <c r="E12" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
-      <c r="I12" s="3" t="s">
-        <v>31</v>
-      </c>
+      <c r="I12" s="3"/>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>34</v>
-      </c>
       <c r="D13" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>102</v>
+        <v>29</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>91</v>
       </c>
       <c r="H13" s="3"/>
-      <c r="I13" s="3" t="s">
-        <v>31</v>
+      <c r="I13" s="3">
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -1000,393 +972,377 @@
         <v>15</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>37</v>
-      </c>
       <c r="E14" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G14" s="3">
         <v>4</v>
       </c>
       <c r="H14" s="3"/>
-      <c r="I14" s="3" t="s">
-        <v>31</v>
+      <c r="I14" s="3">
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="D15" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>41</v>
-      </c>
       <c r="E15" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
-      <c r="I15" s="3" t="s">
-        <v>42</v>
-      </c>
+      <c r="I15" s="3"/>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>46</v>
-      </c>
       <c r="E16" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G16" s="3">
         <v>4</v>
       </c>
       <c r="H16" s="3"/>
-      <c r="I16" s="3" t="s">
-        <v>47</v>
+      <c r="I16" s="3">
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
-      <c r="I17" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
-      <c r="A18" s="3" t="s">
+      <c r="I17" s="3"/>
+    </row>
+    <row r="18" spans="1:9" s="11" customFormat="1">
+      <c r="A18" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G18" s="6">
+        <v>4</v>
+      </c>
+      <c r="H18" s="6"/>
+      <c r="I18" s="6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" s="11" customFormat="1">
+      <c r="A19" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B19" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C19" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D19" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E18" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G18" s="9">
-        <v>4</v>
-      </c>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
-      <c r="A19" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G19" s="9">
-        <v>4</v>
-      </c>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3" t="s">
-        <v>61</v>
+      <c r="E19" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G19" s="6">
+        <v>4</v>
+      </c>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6">
+        <v>4</v>
       </c>
     </row>
     <row r="20" spans="1:9">
       <c r="A20" s="3" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G20" s="3">
         <v>4</v>
       </c>
       <c r="H20" s="3"/>
-      <c r="I20" s="3" t="s">
-        <v>66</v>
+      <c r="I20" s="3">
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" s="3" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G21" s="3">
         <v>4</v>
       </c>
       <c r="H21" s="3"/>
-      <c r="I21" s="3" t="s">
-        <v>70</v>
+      <c r="I21" s="3">
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="3" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
-      <c r="I22" s="3" t="s">
-        <v>31</v>
-      </c>
+      <c r="I22" s="3"/>
     </row>
     <row r="23" spans="1:9">
       <c r="A23" s="3" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
-      <c r="I23" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G24" s="9">
-        <v>4</v>
-      </c>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3" t="s">
-        <v>31</v>
+      <c r="I23" s="3"/>
+    </row>
+    <row r="24" spans="1:9" s="11" customFormat="1">
+      <c r="A24" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G24" s="6">
+        <v>4</v>
+      </c>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6">
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="3" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G25" s="3">
         <v>4</v>
       </c>
       <c r="H25" s="3"/>
-      <c r="I25" s="3" t="s">
-        <v>87</v>
-      </c>
+      <c r="I25" s="3"/>
     </row>
     <row r="26" spans="1:9">
       <c r="A26" s="3" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="3">
         <v>0</v>
       </c>
-      <c r="I26" s="3" t="s">
-        <v>31</v>
-      </c>
+      <c r="I26" s="3"/>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" s="3" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
-      <c r="I27" s="3" t="s">
-        <v>96</v>
-      </c>
+      <c r="I27" s="3"/>
     </row>
     <row r="28" spans="1:9">
       <c r="A28" s="3" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
-      <c r="I28" s="3" t="s">
-        <v>100</v>
-      </c>
+      <c r="I28" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1400,7 +1356,7 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I10 A12:F28 A11:F11 I11 I12:I28" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:I10 A12:F28 A11:F11" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>